<commit_message>
0.19b | agent id complete
</commit_message>
<xml_diff>
--- a/src/data/agent-profiles.xlsx
+++ b/src/data/agent-profiles.xlsx
@@ -11,39 +11,94 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
-  <si>
-    <t>Agent ID</t>
-  </si>
-  <si>
-    <t>Discord ID</t>
-  </si>
-  <si>
-    <t>SHD ID</t>
-  </si>
-  <si>
-    <t>Surname</t>
-  </si>
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Sex</t>
-  </si>
-  <si>
-    <t>Date of Birth</t>
-  </si>
-  <si>
-    <t>Occupational Specialty</t>
-  </si>
-  <si>
-    <t>Date of Activation</t>
-  </si>
-  <si>
-    <t>Deployment Wave</t>
-  </si>
-  <si>
-    <t>Avatar URL</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Agent ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Discord ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>SHD ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Surname</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>First Name</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Sex</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Date of Birth</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Occupational Specialty</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Date of Activation</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Deployment Wave</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Avatar URL</t>
+    </r>
   </si>
   <si>
     <t>391723953283923971</t>
@@ -76,7 +131,9 @@
     <t>534781641516908565</t>
   </si>
   <si>
-    <t>SHD-01-6453722</t>
+    <r>
+      <t>SHD-02-6453722</t>
+    </r>
   </si>
   <si>
     <t>Vivian</t>
@@ -85,6 +142,9 @@
     <t>Blair</t>
   </si>
   <si>
+    <t>05/02/1990</t>
+  </si>
+  <si>
     <t>Safecracker</t>
   </si>
   <si>
@@ -97,7 +157,9 @@
     <t>581519836618948615</t>
   </si>
   <si>
-    <t>SHD-01-1749885</t>
+    <r>
+      <t>SHD-02-1749885</t>
+    </r>
   </si>
   <si>
     <t>Kurov</t>
@@ -584,14 +646,17 @@
       <c r="F3" t="s">
         <v>15</v>
       </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -599,31 +664,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
         <v>27</v>
-      </c>
-      <c r="C4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>